<commit_message>
updated on 25th august
</commit_message>
<xml_diff>
--- a/12613356.xlsx
+++ b/12613356.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d0c5ea7b5c0f020d/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d0c5ea7b5c0f020d/Desktop/CAP 776/CAP-776/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="27" documentId="8_{7FDAD421-8814-4830-A1D8-C9C2A23F8EFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C212CC08-2393-43EC-9D91-7C0A55B19E08}"/>
+  <xr:revisionPtr revIDLastSave="28" documentId="8_{7FDAD421-8814-4830-A1D8-C9C2A23F8EFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DE7F5E37-DFDA-43EE-9939-DC9BCD564FE3}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{24114507-0DC2-48E7-A782-B3DFA67E219B}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="31">
   <si>
     <t>My Data, My Code — Daily Log</t>
   </si>
@@ -126,6 +126,9 @@
   </si>
   <si>
     <t>bored</t>
+  </si>
+  <si>
+    <t>eff3rcvbnm,.</t>
   </si>
 </sst>
 </file>
@@ -298,10 +301,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -885,7 +884,9 @@
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" s="8"/>
-      <c r="B9" s="9"/>
+      <c r="B9" s="9" t="s">
+        <v>30</v>
+      </c>
       <c r="C9" s="9"/>
       <c r="D9" s="9"/>
       <c r="E9" s="9"/>

</xml_diff>